<commit_message>
Security: hide credentials from docs/xlsx and strip sensitive data from CI report
- README.md: no literal credentials; note on htmlextra privacy flags
- xlsx: request bodies use {{valid_login}}/{{valid_password}}/{{invalid_*}} placeholders
- workflow: omitHeaders/omitRequestBodies/omitResponseBodies so token and creds never land in report artifact
- collection: sync test cases with xlsx (39 cases), asserts for silent cases, no hardcoded creds
</commit_message>
<xml_diff>
--- a/RestfulBooker_Тест-кейсы_Баг-репорты.xlsx
+++ b/RestfulBooker_Тест-кейсы_Баг-репорты.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>{"username":"admin","password":"password123"}</t>
+          <t>{"username":"{{valid_login}}","password":"{{valid_password}}"}</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>{"username":"wrong","password":"password123"}</t>
+          <t>{"username":"{{invalid_login}}","password":"{{valid_password}}"}</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>{"username":"admin","password":"wrong"}</t>
+          <t>{"username":"{{valid_login}}","password":"{{invalid_password}}"}</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>{"username":"","password":"password123"}</t>
+          <t>{"username":"","password":"{{valid_password}}"}</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>{"username":"admin","password":""}</t>
+          <t>{"username":"{{valid_login}}","password":""}</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1065,45 +1065,49 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TC-LIST-001</t>
+          <t>TC-BOOK-009</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Get Bookings List</t>
+          <t>Create Booking</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>GET /booking</t>
+          <t>POST /booking</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Без параметров.</t>
+          <t>Malformed JSON body</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; список booking IDs.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>HTTP 400 Bad Request; понятная ошибка парсинга.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>BUG-005; факт: 400 Bad Request (подтверждено).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TC-LIST-002</t>
+          <t>TC-LIST-001</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1123,17 +1127,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>filter по firstname.</t>
+          <t>Без параметров.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; возвращены соответствующие записи.</t>
+          <t>HTTP 200; список booking IDs.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1141,7 +1145,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TC-LIST-003</t>
+          <t>TC-LIST-002</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1166,7 +1170,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>filter по lastname.</t>
+          <t>filter по firstname.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1179,7 +1183,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TC-LIST-004</t>
+          <t>TC-LIST-003</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1194,7 +1198,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1204,12 +1208,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Несуществующий filter.</t>
+          <t>filter по lastname.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; пустой список.</t>
+          <t>HTTP 200; возвращены соответствующие записи.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1217,17 +1221,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TC-GET-001</t>
+          <t>TC-LIST-004</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Get Booking by ID</t>
+          <t>Get Bookings List</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>GET /booking/:id</t>
+          <t>GET /booking</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1237,17 +1241,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Существующий bookingId.</t>
+          <t>filter по checkin и checkout.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; корректное тело бронирования.</t>
+          <t>HTTP 200; возвращены записи в диапазоне дат.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1255,37 +1259,37 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TC-GET-002</t>
+          <t>TC-LIST-005</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Get Booking by ID</t>
+          <t>Get Bookings List</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>GET /booking/:id</t>
+          <t>GET /booking</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Несуществующий bookingId.</t>
+          <t>filter по firstname, lastname, checkin и checkout одновременно.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>HTTP 404 Not Found.</t>
+          <t>HTTP 200; возвращены соответствующие записи.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1293,17 +1297,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TC-GET-003</t>
+          <t>TC-LIST-006</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Get Booking by ID</t>
+          <t>Get Bookings List</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>GET /booking/:id</t>
+          <t>GET /booking</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1318,12 +1322,12 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Некорректный ID.</t>
+          <t>Несуществующий firstname (несуществующий filter).</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>HTTP 404/400 согласно контракту.</t>
+          <t>HTTP 200; пустой список.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1331,60 +1335,64 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TC-PUT-001</t>
+          <t>TC-LIST-007</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Update Booking</t>
+          <t>Get Bookings List</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>PUT /booking/:id</t>
+          <t>GET /booking</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Существующий bookingId + полный валидный payload + token.</t>
+          <t>Невалидная дата в filter (checkin=abc).</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; данные полностью обновлены.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>HTTP 400; ошибка валидации.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Факт: 500 — толерантно зафиксировано в коллекции (баг API).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TC-PUT-002</t>
+          <t>TC-GET-001</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Update Booking</t>
+          <t>Get Booking by ID</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>PUT /booking/:id</t>
+          <t>GET /booking/:id</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1394,12 +1402,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Без Authorization.</t>
+          <t>Существующий bookingId.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401/403; обновление не выполнено.</t>
+          <t>HTTP 200; корректное тело бронирования.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1407,17 +1415,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TC-PUT-003</t>
+          <t>TC-GET-002</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Update Booking</t>
+          <t>Get Booking by ID</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>PUT /booking/:id</t>
+          <t>GET /booking/:id</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1432,7 +1440,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Несуществующий bookingId + валидная авторизация.</t>
+          <t>Несуществующий bookingId.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1440,26 +1448,22 @@
           <t>HTTP 404 Not Found.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>BUG-006</t>
-        </is>
-      </c>
+      <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TC-PUT-004</t>
+          <t>TC-GET-003</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Update Booking</t>
+          <t>Get Booking by ID</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>PUT /booking/:id</t>
+          <t>GET /booking/:id</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1469,29 +1473,25 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Неполный/некорректный payload.</t>
+          <t>Некорректный ID.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400/422, а не 500.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>BUG-005</t>
-        </is>
-      </c>
+          <t>HTTP 404/400 согласно контракту.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TC-PUT-005</t>
+          <t>TC-PUT-001</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1506,22 +1506,22 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Некорректный token.</t>
+          <t>Существующий bookingId + полный валидный payload + token.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401/403; обновление не выполнено.</t>
+          <t>HTTP 200; данные полностью обновлены.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1529,22 +1529,22 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TC-PATCH-001</t>
+          <t>TC-PUT-002</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Partial Update</t>
+          <t>Update Booking</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>PATCH /booking/:id</t>
+          <t>PUT /booking/:id</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1554,12 +1554,12 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Существующий bookingId + одно изменяемое поле + token.</t>
+          <t>Без Authorization.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; изменено только указанное поле.</t>
+          <t>HTTP 401/403; обновление не выполнено.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1567,22 +1567,22 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TC-PATCH-002</t>
+          <t>TC-PUT-003</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Partial Update</t>
+          <t>Update Booking</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>PATCH /booking/:id</t>
+          <t>PUT /booking/:id</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1592,30 +1592,34 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Существующий bookingId + несколько полей + token.</t>
+          <t>Несуществующий bookingId + валидная авторизация.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; изменены только указанные поля.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>HTTP 404 Not Found.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>BUG-006</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TC-PATCH-003</t>
+          <t>TC-PUT-004</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Partial Update</t>
+          <t>Update Booking</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>PATCH /booking/:id</t>
+          <t>PUT /booking/:id</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1630,30 +1634,34 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Без Authorization.</t>
+          <t>Неполный/некорректный payload.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401/403; обновление не выполнено.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
+          <t>HTTP 400/422, а не 500.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>BUG-005</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>TC-PATCH-004</t>
+          <t>TC-PUT-005</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Partial Update</t>
+          <t>Update Booking</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>PATCH /booking/:id</t>
+          <t>PUT /booking/:id</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1668,34 +1676,30 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Несуществующий bookingId + token.</t>
+          <t>Некорректный token.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>HTTP 404 Not Found.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>BUG-006</t>
-        </is>
-      </c>
+          <t>HTTP 401/403; обновление не выполнено.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TC-DELETE-001</t>
+          <t>TC-PATCH-001</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Delete Booking</t>
+          <t>Partial Update</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>DELETE /booking/:id</t>
+          <t>PATCH /booking/:id</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1710,54 +1714,50 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Существующий bookingId + token.</t>
+          <t>Существующий bookingId + одно изменяемое поле + token.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>HTTP 201/200 согласно контракту; запись удалена.</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Запускать первым в папке; после удаления GET должен вернуть 404.</t>
-        </is>
-      </c>
+          <t>HTTP 200; изменено только указанное поле.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TC-DELETE-002</t>
+          <t>TC-PATCH-002</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Delete Booking</t>
+          <t>Partial Update</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>DELETE /booking/:id</t>
+          <t>PATCH /booking/:id</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Без Authorization.</t>
+          <t>Существующий bookingId + несколько полей + token.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401/403; удаление не выполнено.</t>
+          <t>HTTP 200; изменены только указанные поля.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -1765,17 +1765,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TC-DELETE-003</t>
+          <t>TC-PATCH-003</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Delete Booking</t>
+          <t>Partial Update</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>DELETE /booking/:id</t>
+          <t>PATCH /booking/:id</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1785,39 +1785,35 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Несуществующий bookingId + token.</t>
+          <t>Без Authorization.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>HTTP 404 Not Found.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>BUG-006</t>
-        </is>
-      </c>
+          <t>HTTP 401/403; обновление не выполнено.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TC-DELETE-004</t>
+          <t>TC-PATCH-004</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Delete Booking</t>
+          <t>Partial Update</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>DELETE /booking/:id</t>
+          <t>PATCH /booking/:id</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1837,7 +1833,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>HTTP 404 Not Found; повторное удаление не должно приводить к 500.</t>
+          <t>HTTP 404 Not Found.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1849,40 +1845,250 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>TC-PATCH-005</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Partial Update</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /booking/:id</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Пустой объект {}</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400/422; ошибка валидации.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Факт: 200 OK, тело бронирования без изменений (зафиксировано в коллекции).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-DELETE-001</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Delete Booking</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /booking/:id</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Существующий bookingId + token.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 201/200 согласно контракту; запись удалена.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Запускать первым в папке; после удаления GET должен вернуть 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-DELETE-002</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Delete Booking</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /booking/:id</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Без Authorization.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 401/403; удаление не выполнено.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TC-DELETE-003</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Delete Booking</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /booking/:id</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Несуществующий bookingId + token.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>BUG-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TC-DELETE-004</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Delete Booking</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /booking/:id</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>BookingId уже удалённой ранее брони + token.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found; повторное удаление не должно приводить к 500.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>BUG-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>TC-HEALTH-001</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Health Check</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>GET /ping</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Без параметров.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>HTTP 201/200; сервис доступен.</t>
         </is>
       </c>
-      <c r="H35" s="2" t="n"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>В коллекции кейс именуется TC-PING-001.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H35"/>
@@ -2011,7 +2217,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"username":"wrong","password":"password123"}</t>
+          <t>{"username":"{{invalid_login}}","password":"{{valid_password}}"}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -2145,7 +2351,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 OK; бронирование создано с сохранением некорректного типа значения.</t>
+          <t>HTTP 200 OK; бронирование создано, totalprice сохранён как null (некорректный ввод не отвергается и не нормализуется).</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add QA-middle asserts; sync xlsx/README docs with actual API behavior
Коллекция (+27 pm.test, 164->191): echo-контракт создания, CRUD read-back (deep-equal), персистентность PUT/PATCH/DELETE через повторный GET (pm.sendRequest), неизменность данных после 403/400, уникальность и позитивность bookingid, Content-Type, формат token, точные тела ошибок (500 Internal Server Error / 400 Bad Request); TC-PATCH-005 (empty patch) покрыт ассертами (no-op 200).

Новый BUG-007: фильтр /booking по точным датам существующей брони -> пустой массив (TC-LIST-004/005 - только структурные ассерты, поведение недетерминировано).

xlsx: синхронизировано 25 ячеек тест-кейсов, BUG-001 расширена на TC-AUTH-002..005, BUG-005/006 подтверждены прогонами (400 Bad Request / 405 Method Not Allowed), добавлен BUG-007. README: строка BUG-007 в таблице багов + пункт про middle-проверки.

Валидация: Newman 191 assertion / 0 failed (51 запрос, live API).
</commit_message>
<xml_diff>
--- a/RestfulBooker_Тест-кейсы_Баг-репорты.xlsx
+++ b/RestfulBooker_Тест-кейсы_Баг-репорты.xlsx
@@ -570,7 +570,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Setup: сохранить token.</t>
+          <t>Setup: сохранить token. Middle: формат token (10-32 алфанумерных символа), Content-Type: application/json.</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,11 @@
           <t>HTTP 401/403; ошибка; токен отсутствует.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>BUG-001</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -682,7 +686,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>{"username":"","password":"{{valid_password}}"}</t>
+          <t>Пустой объект {}</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -690,7 +694,11 @@
           <t>HTTP 400/401/403; ошибка валидации/аутентификации.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>BUG-001; факт: HTTP 200 + {"reason":"Bad credentials"} (подтверждено).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -728,7 +736,11 @@
           <t>HTTP 400/401/403; ошибка; токен отсутствует.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>BUG-001</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -768,7 +780,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Setup: сохранить bookingId.</t>
+          <t>Setup: сохранить bookingId. Middle: echo — booking deep-equal payload; bookingid — целое &gt; 0; Content-Type JSON.</t>
         </is>
       </c>
     </row>
@@ -890,7 +902,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>BUG-005</t>
+          <t>BUG-005; факт: HTTP 500 + тело "Internal Server Error" (подтверждено).</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1028,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>BUG-005</t>
+          <t>BUG-005; факт: HTTP 500 + тело "Internal Server Error" (подтверждено).</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1070,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>BUG-005</t>
+          <t>BUG-005; факт: HTTP 500 + тело "Internal Server Error" (подтверждено).</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1152,11 @@
           <t>HTTP 200; список booking IDs.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Middle: все bookingid — целые &gt; 0 и уникальны в списке.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1178,7 +1194,11 @@
           <t>HTTP 200; возвращены соответствующие записи.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Middle: результат содержит bookingId из Setup (TC-BOOK-001).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1216,7 +1236,11 @@
           <t>HTTP 200; возвращены соответствующие записи.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Middle: результат содержит bookingId из Setup (TC-BOOK-001).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1254,7 +1278,11 @@
           <t>HTTP 200; возвращены записи в диапазоне дат.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>BUG-007: точный датный фильтр возвращает пустой массив (подтверждено).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1292,7 +1320,11 @@
           <t>HTTP 200; возвращены соответствующие записи.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>BUG-007: комбинированный фильтр с точными датами возвращает пустой массив (подтверждено).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1410,7 +1442,11 @@
           <t>HTTP 200; корректное тело бронирования.</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Middle: тело = payload из TC-BOOK-001 (deep-equal всех полей); Content-Type JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1524,7 +1560,11 @@
           <t>HTTP 200; данные полностью обновлены.</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Middle: персистентность — повторный GET возвращает обновлённые данные.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1562,7 +1602,11 @@
           <t>HTTP 401/403; обновление не выполнено.</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Middle: после отказа GET подтверждает, что данные не изменились.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1644,7 +1688,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>BUG-005</t>
+          <t>BUG-005; факт: HTTP 400 "Bad Request"; middle: после ошибки данные не повреждены (GET).</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1728,11 @@
           <t>HTTP 401/403; обновление не выполнено.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Middle: после отказа GET подтверждает, что данные не изменились.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1722,7 +1770,11 @@
           <t>HTTP 200; изменено только указанное поле.</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Middle: персистентность — GET подтверждает обновление firstname и сохранность остальных полей.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1760,7 +1812,11 @@
           <t>HTTP 200; изменены только указанные поля.</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Middle: персистентность — GET подтверждает обновление totalprice/additionalneeds и сохранность firstname.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1798,7 +1854,11 @@
           <t>HTTP 401/403; обновление не выполнено.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Middle: после отказа GET подтверждает, что данные не изменились.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1922,7 +1982,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Запускать первым в папке; после удаления GET должен вернуть 404.</t>
+          <t>Запускать первым в папке; после удаления GET должен вернуть 404 (автоматизировано middle-ассертом).</t>
         </is>
       </c>
     </row>
@@ -1962,7 +2022,11 @@
           <t>HTTP 401/403; удаление не выполнено.</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Внимание: в коллекции бронь уже удалена на TC-DELETE-001; проверяется отказ авторизации (403 до проверки существования).</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2086,7 +2150,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>В коллекции кейс именуется TC-PING-001.</t>
+          <t>В коллекции кейс именуется TC-PING-001. Факт: 201 + Content-Type: text/plain.</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2232,7 +2296,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>TC-AUTH-002</t>
+          <t>TC-AUTH-002, TC-AUTH-003, TC-AUTH-004, TC-AUTH-005</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2475,7 +2539,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Сервис может вернуть HTTP 500 Internal Server Error и/или обобщенное тело ответа.</t>
+          <t>POST /booking с {}, без firstname или без lastname → HTTP 500 + тело "Internal Server Error"; malformed JSON и PUT /booking/:id без lastname → HTTP 400 "Bad Request" (подтверждено прогоном коллекции).</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -2490,7 +2554,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Требует подтверждения запуском коллекции, поскольку поведение публичного сервиса может изменяться.</t>
+          <t>Подтверждено прогонами коллекции; поведение публичного сервиса может изменяться.</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2601,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>В зависимости от метода сервис может вернуть HTTP 405 или 500.</t>
+          <t>Подтверждено прогоном коллекции: PUT, PATCH и DELETE несуществующего bookingId → HTTP 405 Method Not Allowed.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -2552,7 +2616,69 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Требует подтверждения запуском коллекции, поскольку поведение публичного сервиса может изменяться.</t>
+          <t>Подтверждено прогонами коллекции (405 для всех трёх методов); поведение публичного сервиса может изменяться.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>BUG-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Фильтр /booking по точным датам существующей брони возвращает пустой результат</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>GET /booking</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>checkin=2026-04-09, checkout=2026-04-15 (точные даты существующей брони)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200; список содержит бронь с этими датами.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200; пустой массив [] — бронь с точно такими датами не находится.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>TC-LIST-004, TC-LIST-005</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Фильтрация по датам фактически недоступна; клиенты получают ложный ответ «броней нет».</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено пробой и прогоном коллекции; в коллекции структура ответа проверяется без датного ассерта.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync xlsx test cases & bug reports with collection: add BUG-008..012, update BUG-006 (DELETE->403)
</commit_message>
<xml_diff>
--- a/RestfulBooker_Тест-кейсы_Баг-репорты.xlsx
+++ b/RestfulBooker_Тест-кейсы_Баг-репорты.xlsx
@@ -1402,7 +1402,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Факт: 500 — толерантно зафиксировано в коллекции (баг API).</t>
+          <t>Факт: 500 — толерантно зафиксировано в коллекции (баг API). BUG-011.</t>
         </is>
       </c>
     </row>
@@ -1519,10 +1519,14 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>HTTP 404/400 согласно контракту.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
+          <t>HTTP 400 Bad Request (контракт); понятная ошибка.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Факт: HTTP 404 Not Found (вместо 400); BUG-010.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1940,7 +1944,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Факт: 200 OK, тело бронирования без изменений (зафиксировано в коллекции).</t>
+          <t>Факт: 200 OK, тело бронирования без изменений (зафиксировано в коллекции). BUG-009.</t>
         </is>
       </c>
     </row>
@@ -1977,12 +1981,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>HTTP 201/200 согласно контракту; запись удалена.</t>
+          <t>HTTP 204 No Content (контракт); запись удалена.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Запускать первым в папке; после удаления GET должен вернуть 404 (автоматизировано middle-ассертом).</t>
+          <t>Запускать первым в папке; после удаления GET должен вернуть 404 (автоматизировано middle-ассертом). Факт: HTTP 201 Created + тело "Created" (вместо 204); BUG-008.</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2070,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>BUG-006</t>
+          <t>BUG-006 (07.09.2026: DELETE несуществующей/удалённой брони возвращал 403).</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2112,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>BUG-006</t>
+          <t>BUG-006 (07.09.2026: DELETE несуществующей/удалённой брони возвращал 403).</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2154,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>В коллекции кейс именуется TC-PING-001. Факт: 201 + Content-Type: text/plain.</t>
+          <t>В коллекции кейс именуется TC-PING-001. Факт: 201 + Content-Type: text/plain. BUG-012.</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2601,7 +2605,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Подтверждено прогоном коллекции: PUT, PATCH и DELETE несуществующего bookingId → HTTP 405 Method Not Allowed.</t>
+          <t>PUT и PATCH несуществующего bookingId -&gt; HTTP 405 Method Not Allowed (подтверждено прогонами коллекции); в прогонах 07.09.2026 DELETE несуществующего/уже удалённого bookingId возвращал HTTP 403.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -2616,7 +2620,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Подтверждено прогонами коллекции (405 для всех трёх методов); поведение публичного сервиса может изменяться.</t>
+          <t>Подтверждено прогонами коллекции: PUT/PATCH -&gt; 405; DELETE -&gt; 403 (прогоны 07.09.2026), ранее фиксировался 405 для всех трёх методов.</t>
         </is>
       </c>
     </row>
@@ -2679,6 +2683,316 @@
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Подтверждено пробой и прогоном коллекции; в коллекции структура ответа проверяется без датного ассерта.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>BUG-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>DELETE успешной брони возвращает 201 Created с телом</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /booking/:id</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Существующий bookingId + валидный token</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 204 No Content без тела.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created; тело "Created".</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>TC-DELETE-001</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Отличие от REST-конвенций; потребители, ожидающие 204/пустого тела, должны учитывать нестандартный статус.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено прогоном коллекции 07.09.2026; фактический ассерт коллекции ждёт 201, Contract-проверка — 204.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>BUG-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>PATCH с пустым телом {} не отклоняется</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /booking/:id</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>bookingId + {} (пустое тело) + валидный token</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400/422; ошибка валидации; данные не изменяются.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK; тело — текущее состояние брони без изменений (no-op).</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>TC-PATCH-005</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Отсутствует ранняя валидация пустого тела; клиент не получает сигнала о пустом запросе.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено прогоном коллекции; контрактный ассерт ожидает 400, фактически 200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>BUG-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>GET /booking/:id с не-числовым ID возвращает 404 вместо 400</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>GET /booking/:id</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>bookingId=abc</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request; понятное сообщение об ошибке.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found; тело "Not Found".</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>TC-GET-003</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Некорректный формат ID трактуется как отсутствующий ресурс; контракт не различает эти случаи.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено прогоном коллекции.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>BUG-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>GET /booking с невалидной датой фильтра возвращает HTTP 500</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>GET /booking</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>checkin=not-a-date</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request; ошибка валидации.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 500; тело "Internal Server Error".</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>TC-LIST-007</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Ошибка клиентского ввода классифицируется как серверная; шум в мониторинге и алертах.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено прогоном коллекции; в коллекции ассерт допускает [200,400,500] с контрактной проверкой на 400.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>BUG-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>GET /ping возвращает HTTP 201 вместо 200</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>GET /ping</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Без параметров</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created; тело "Created"; Content-Type: text/plain.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>TC-PING-001 (в xlsx — TC-HEALTH-001)</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Нестандартный статус для health-эндпоинта; может нарушить мониторинг, ожидающий заданный статус.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено прогоном коллекции; контрактный ассерт ожидает 200.</t>
         </is>
       </c>
     </row>

</xml_diff>